<commit_message>
stockInfo-list and log finish
</commit_message>
<xml_diff>
--- a/docs/【DIGITAL OJT】WBS.xlsx
+++ b/docs/【DIGITAL OJT】WBS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DIGITALOJT\digital-ojt-development-cause-DroneInventorySystem\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F96B42F-D5CE-4636-A4F5-4AD97EEFDCB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF7D336E-BEB3-4E9A-B1FF-CC319252A505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WBS" sheetId="1" r:id="rId1"/>
@@ -1736,7 +1736,7 @@
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="50">
+  <dxfs count="17">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1744,272 +1744,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFBFBFBF"/>
-          <bgColor rgb="FFBFBFBF"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2353,14 +2087,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:DP276"/>
-  <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="7" width="5" customWidth="1"/>
-    <col min="8" max="8" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="61" width="3.44140625" customWidth="1"/>
-    <col min="62" max="63" width="3.44140625" style="100" customWidth="1"/>
-    <col min="64" max="119" width="3.44140625" customWidth="1"/>
+    <col min="10" max="61" width="3.42578125" customWidth="1"/>
+    <col min="62" max="63" width="3.42578125" style="100" customWidth="1"/>
+    <col min="64" max="119" width="3.42578125" customWidth="1"/>
     <col min="120" max="120" width="5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -14277,7 +14011,7 @@
       <c r="AR92" s="21"/>
       <c r="AS92" s="20"/>
       <c r="AT92" s="20"/>
-      <c r="AU92" s="69"/>
+      <c r="AU92" s="75"/>
       <c r="AV92" s="69"/>
       <c r="AW92" s="69"/>
       <c r="AX92" s="21"/>
@@ -14526,7 +14260,7 @@
       <c r="AS94" s="20"/>
       <c r="AT94" s="20"/>
       <c r="AU94" s="69"/>
-      <c r="AV94" s="69"/>
+      <c r="AV94" s="75"/>
       <c r="AW94" s="69"/>
       <c r="AX94" s="21"/>
       <c r="AY94" s="21"/>
@@ -14775,7 +14509,7 @@
       <c r="AT96" s="20"/>
       <c r="AU96" s="20"/>
       <c r="AV96" s="20"/>
-      <c r="AW96" s="20"/>
+      <c r="AW96" s="75"/>
       <c r="AX96" s="21"/>
       <c r="AY96" s="21"/>
       <c r="AZ96" s="69"/>
@@ -15026,7 +14760,7 @@
       <c r="AW98" s="20"/>
       <c r="AX98" s="21"/>
       <c r="AY98" s="21"/>
-      <c r="AZ98" s="69"/>
+      <c r="AZ98" s="75"/>
       <c r="BA98" s="69"/>
       <c r="BB98" s="69"/>
       <c r="BC98" s="69"/>
@@ -15275,7 +15009,7 @@
       <c r="AX100" s="21"/>
       <c r="AY100" s="21"/>
       <c r="AZ100" s="69"/>
-      <c r="BA100" s="69"/>
+      <c r="BA100" s="75"/>
       <c r="BB100" s="69"/>
       <c r="BC100" s="69"/>
       <c r="BD100" s="20"/>
@@ -36935,87 +36669,87 @@
   </mergeCells>
   <phoneticPr fontId="10"/>
   <conditionalFormatting sqref="J7">
-    <cfRule type="expression" dxfId="33" priority="15">
+    <cfRule type="expression" dxfId="16" priority="15">
       <formula>OR(J4="土", J4="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J9:J12">
-    <cfRule type="expression" dxfId="32" priority="13">
+    <cfRule type="expression" dxfId="15" priority="13">
       <formula>OR(J6="土", J6="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J161">
-    <cfRule type="expression" dxfId="31" priority="17">
+    <cfRule type="expression" dxfId="14" priority="17">
       <formula>OR(#REF!="土", #REF!="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J7:DO8 AA52:DO52 J9:Y64 AA55:DO58 Z59:DO62 J65:DO66 J137:BN137 BP137:DO137 J138:DO269 J72:DO136">
-    <cfRule type="expression" dxfId="30" priority="16">
+    <cfRule type="expression" dxfId="13" priority="16">
       <formula>OR(J$6="土", J$6="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB51:DO51 Z51:Z52 J71:AN71 AP71:DO71 Z9:DO48 Z55:Z56 Z53:DO54 Z50:DO50 AA49:DO49 J67:AL67 AO67:DO67 J68:DO70">
-    <cfRule type="expression" dxfId="29" priority="14">
+    <cfRule type="expression" dxfId="12" priority="14">
       <formula>OR(J$6="土", J$6="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA51">
-    <cfRule type="expression" dxfId="28" priority="12">
+    <cfRule type="expression" dxfId="11" priority="12">
       <formula>OR(AA$6="土", AA$6="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO71">
-    <cfRule type="expression" dxfId="27" priority="11">
+    <cfRule type="expression" dxfId="10" priority="11">
       <formula>OR(AO$6="土", AO$6="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J21:J22">
-    <cfRule type="expression" dxfId="26" priority="10">
+    <cfRule type="expression" dxfId="9" priority="10">
       <formula>OR(J18="土", J18="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J25:J26">
-    <cfRule type="expression" dxfId="25" priority="9">
+    <cfRule type="expression" dxfId="8" priority="9">
       <formula>OR(J22="土", J22="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J31:J32">
-    <cfRule type="expression" dxfId="24" priority="8">
+    <cfRule type="expression" dxfId="7" priority="8">
       <formula>OR(J28="土", J28="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25">
-    <cfRule type="expression" dxfId="23" priority="7">
+    <cfRule type="expression" dxfId="6" priority="7">
       <formula>OR(K22="土", K22="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K11">
-    <cfRule type="expression" dxfId="22" priority="6">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>OR(K8="土", K8="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K9">
-    <cfRule type="expression" dxfId="21" priority="5">
+    <cfRule type="expression" dxfId="4" priority="5">
       <formula>OR(K6="土", K6="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z63:DO64">
-    <cfRule type="expression" dxfId="20" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>OR(Z$6="土", Z$6="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z49">
-    <cfRule type="expression" dxfId="19" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>OR(Z$6="土", Z$6="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AM67:AN67">
-    <cfRule type="expression" dxfId="18" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>OR(AM$6="土", AM$6="日")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5:DO5">
-    <cfRule type="timePeriod" dxfId="17" priority="1" timePeriod="today">
+    <cfRule type="timePeriod" dxfId="0" priority="1" timePeriod="today">
       <formula>FLOOR(J5,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>